<commit_message>
Add multi-month data, CM/DUoS benchmarks, invoice reconciliation, and technical docs
- Add Nov 2025, Dec 2025, Jan 2026 master and optimized data files
- Integrate Capacity Market and DUoS actuals into benchmark and executive comparison tables
- Add dynamic IAR loading from Excel for benchmark Section 2
- Remove Gap metric cards from benchmark Key Performance Metrics
- Add invoice loader, reconciler, and invoice analysis page
- Add monthly checklist page
- Add raw EMR settlement CSVs and Hartree DUoS invoices
- Generate APD Technical Reference (DOCX) for DoublU development team
- Generate Optimisation Validation document (DOCX + PDF) with Jan 2026 worked examples
- Add market data subscription docs (DE/NL, UK)
- Update data cleaning pipeline (loader, transformer, init)
- Update requirements.txt with new dependencies

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/raw/october2025/export-01_10_2025-02_11_2025 (1).xlsx
+++ b/raw/october2025/export-01_10_2025-02_11_2025 (1).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\bess-dashboard\raw\october2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAC8A73E-5491-4E50-B90B-02E5425BACE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD3F7735-84B0-4099-AD64-8C7E50665FFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13761,3117 +13761,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:lineChart>
-        <c:grouping val="standard"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet0!$A$145:$A$287</c:f>
-              <c:strCache>
-                <c:ptCount val="143"/>
-                <c:pt idx="0">
-                  <c:v>02/10/2025 00:00:00</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>02/10/2025 00:10:00</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>02/10/2025 00:20:00</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>02/10/2025 00:30:00</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>02/10/2025 00:40:00</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>02/10/2025 00:50:00</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>02/10/2025 01:00:00</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>02/10/2025 01:10:00</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>02/10/2025 01:20:00</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>02/10/2025 01:30:00</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>02/10/2025 01:40:00</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>02/10/2025 01:50:00</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>02/10/2025 02:00:00</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>02/10/2025 02:10:00</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>02/10/2025 02:20:00</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>02/10/2025 02:30:00</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>02/10/2025 02:40:00</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>02/10/2025 02:50:00</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>02/10/2025 03:00:00</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>02/10/2025 03:10:00</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>02/10/2025 03:20:00</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>02/10/2025 03:30:00</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>02/10/2025 03:40:00</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>02/10/2025 03:50:00</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>02/10/2025 04:00:00</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>02/10/2025 04:10:00</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>02/10/2025 04:20:00</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>02/10/2025 04:30:00</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>02/10/2025 04:40:00</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>02/10/2025 04:50:00</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>02/10/2025 05:00:00</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>02/10/2025 05:10:00</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>02/10/2025 05:20:00</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>02/10/2025 05:30:00</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>02/10/2025 05:40:00</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>02/10/2025 05:50:00</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>02/10/2025 06:00:00</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>02/10/2025 06:10:00</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>02/10/2025 06:20:00</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>02/10/2025 06:30:00</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>02/10/2025 06:40:00</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>02/10/2025 06:50:00</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>02/10/2025 07:00:00</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>02/10/2025 07:10:00</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>02/10/2025 07:20:00</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>02/10/2025 07:30:00</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>02/10/2025 07:40:00</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>02/10/2025 07:50:00</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>02/10/2025 08:00:00</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>02/10/2025 08:10:00</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>02/10/2025 08:20:00</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>02/10/2025 08:30:00</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>02/10/2025 08:40:00</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>02/10/2025 08:50:00</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>02/10/2025 09:00:00</c:v>
-                </c:pt>
-                <c:pt idx="55">
-                  <c:v>02/10/2025 09:10:00</c:v>
-                </c:pt>
-                <c:pt idx="56">
-                  <c:v>02/10/2025 09:20:00</c:v>
-                </c:pt>
-                <c:pt idx="57">
-                  <c:v>02/10/2025 09:30:00</c:v>
-                </c:pt>
-                <c:pt idx="58">
-                  <c:v>02/10/2025 09:40:00</c:v>
-                </c:pt>
-                <c:pt idx="59">
-                  <c:v>02/10/2025 09:50:00</c:v>
-                </c:pt>
-                <c:pt idx="60">
-                  <c:v>02/10/2025 10:00:00</c:v>
-                </c:pt>
-                <c:pt idx="61">
-                  <c:v>02/10/2025 10:10:00</c:v>
-                </c:pt>
-                <c:pt idx="62">
-                  <c:v>02/10/2025 10:20:00</c:v>
-                </c:pt>
-                <c:pt idx="63">
-                  <c:v>02/10/2025 10:30:00</c:v>
-                </c:pt>
-                <c:pt idx="64">
-                  <c:v>02/10/2025 10:40:00</c:v>
-                </c:pt>
-                <c:pt idx="65">
-                  <c:v>02/10/2025 10:50:00</c:v>
-                </c:pt>
-                <c:pt idx="66">
-                  <c:v>02/10/2025 11:00:00</c:v>
-                </c:pt>
-                <c:pt idx="67">
-                  <c:v>02/10/2025 11:10:00</c:v>
-                </c:pt>
-                <c:pt idx="68">
-                  <c:v>02/10/2025 11:20:00</c:v>
-                </c:pt>
-                <c:pt idx="69">
-                  <c:v>02/10/2025 11:30:00</c:v>
-                </c:pt>
-                <c:pt idx="70">
-                  <c:v>02/10/2025 11:40:00</c:v>
-                </c:pt>
-                <c:pt idx="71">
-                  <c:v>02/10/2025 11:50:00</c:v>
-                </c:pt>
-                <c:pt idx="72">
-                  <c:v>02/10/2025 12:00:00</c:v>
-                </c:pt>
-                <c:pt idx="73">
-                  <c:v>02/10/2025 12:10:00</c:v>
-                </c:pt>
-                <c:pt idx="74">
-                  <c:v>02/10/2025 12:20:00</c:v>
-                </c:pt>
-                <c:pt idx="75">
-                  <c:v>02/10/2025 12:30:00</c:v>
-                </c:pt>
-                <c:pt idx="76">
-                  <c:v>02/10/2025 12:40:00</c:v>
-                </c:pt>
-                <c:pt idx="77">
-                  <c:v>02/10/2025 12:50:00</c:v>
-                </c:pt>
-                <c:pt idx="78">
-                  <c:v>02/10/2025 13:00:00</c:v>
-                </c:pt>
-                <c:pt idx="79">
-                  <c:v>02/10/2025 13:10:00</c:v>
-                </c:pt>
-                <c:pt idx="80">
-                  <c:v>02/10/2025 13:20:00</c:v>
-                </c:pt>
-                <c:pt idx="81">
-                  <c:v>02/10/2025 13:30:00</c:v>
-                </c:pt>
-                <c:pt idx="82">
-                  <c:v>02/10/2025 13:40:00</c:v>
-                </c:pt>
-                <c:pt idx="83">
-                  <c:v>02/10/2025 13:50:00</c:v>
-                </c:pt>
-                <c:pt idx="84">
-                  <c:v>02/10/2025 14:00:00</c:v>
-                </c:pt>
-                <c:pt idx="85">
-                  <c:v>02/10/2025 14:10:00</c:v>
-                </c:pt>
-                <c:pt idx="86">
-                  <c:v>02/10/2025 14:20:00</c:v>
-                </c:pt>
-                <c:pt idx="87">
-                  <c:v>02/10/2025 14:30:00</c:v>
-                </c:pt>
-                <c:pt idx="88">
-                  <c:v>02/10/2025 14:40:00</c:v>
-                </c:pt>
-                <c:pt idx="89">
-                  <c:v>02/10/2025 14:50:00</c:v>
-                </c:pt>
-                <c:pt idx="90">
-                  <c:v>02/10/2025 15:00:00</c:v>
-                </c:pt>
-                <c:pt idx="91">
-                  <c:v>02/10/2025 15:10:00</c:v>
-                </c:pt>
-                <c:pt idx="92">
-                  <c:v>02/10/2025 15:20:00</c:v>
-                </c:pt>
-                <c:pt idx="93">
-                  <c:v>02/10/2025 15:30:00</c:v>
-                </c:pt>
-                <c:pt idx="94">
-                  <c:v>02/10/2025 15:40:00</c:v>
-                </c:pt>
-                <c:pt idx="95">
-                  <c:v>02/10/2025 15:50:00</c:v>
-                </c:pt>
-                <c:pt idx="96">
-                  <c:v>02/10/2025 16:00:00</c:v>
-                </c:pt>
-                <c:pt idx="97">
-                  <c:v>02/10/2025 16:10:00</c:v>
-                </c:pt>
-                <c:pt idx="98">
-                  <c:v>02/10/2025 16:20:00</c:v>
-                </c:pt>
-                <c:pt idx="99">
-                  <c:v>02/10/2025 16:30:00</c:v>
-                </c:pt>
-                <c:pt idx="100">
-                  <c:v>02/10/2025 16:40:00</c:v>
-                </c:pt>
-                <c:pt idx="101">
-                  <c:v>02/10/2025 16:50:00</c:v>
-                </c:pt>
-                <c:pt idx="102">
-                  <c:v>02/10/2025 17:00:00</c:v>
-                </c:pt>
-                <c:pt idx="103">
-                  <c:v>02/10/2025 17:10:00</c:v>
-                </c:pt>
-                <c:pt idx="104">
-                  <c:v>02/10/2025 17:20:00</c:v>
-                </c:pt>
-                <c:pt idx="105">
-                  <c:v>02/10/2025 17:30:00</c:v>
-                </c:pt>
-                <c:pt idx="106">
-                  <c:v>02/10/2025 17:40:00</c:v>
-                </c:pt>
-                <c:pt idx="107">
-                  <c:v>02/10/2025 17:50:00</c:v>
-                </c:pt>
-                <c:pt idx="108">
-                  <c:v>02/10/2025 18:00:00</c:v>
-                </c:pt>
-                <c:pt idx="109">
-                  <c:v>02/10/2025 18:10:00</c:v>
-                </c:pt>
-                <c:pt idx="110">
-                  <c:v>02/10/2025 18:20:00</c:v>
-                </c:pt>
-                <c:pt idx="111">
-                  <c:v>02/10/2025 18:30:00</c:v>
-                </c:pt>
-                <c:pt idx="112">
-                  <c:v>02/10/2025 18:40:00</c:v>
-                </c:pt>
-                <c:pt idx="113">
-                  <c:v>02/10/2025 18:50:00</c:v>
-                </c:pt>
-                <c:pt idx="114">
-                  <c:v>02/10/2025 19:00:00</c:v>
-                </c:pt>
-                <c:pt idx="115">
-                  <c:v>02/10/2025 19:10:00</c:v>
-                </c:pt>
-                <c:pt idx="116">
-                  <c:v>02/10/2025 19:20:00</c:v>
-                </c:pt>
-                <c:pt idx="117">
-                  <c:v>02/10/2025 19:30:00</c:v>
-                </c:pt>
-                <c:pt idx="118">
-                  <c:v>02/10/2025 19:40:00</c:v>
-                </c:pt>
-                <c:pt idx="119">
-                  <c:v>02/10/2025 19:50:00</c:v>
-                </c:pt>
-                <c:pt idx="120">
-                  <c:v>02/10/2025 20:00:00</c:v>
-                </c:pt>
-                <c:pt idx="121">
-                  <c:v>02/10/2025 20:10:00</c:v>
-                </c:pt>
-                <c:pt idx="122">
-                  <c:v>02/10/2025 20:20:00</c:v>
-                </c:pt>
-                <c:pt idx="123">
-                  <c:v>02/10/2025 20:30:00</c:v>
-                </c:pt>
-                <c:pt idx="124">
-                  <c:v>02/10/2025 20:40:00</c:v>
-                </c:pt>
-                <c:pt idx="125">
-                  <c:v>02/10/2025 20:50:00</c:v>
-                </c:pt>
-                <c:pt idx="126">
-                  <c:v>02/10/2025 21:00:00</c:v>
-                </c:pt>
-                <c:pt idx="127">
-                  <c:v>02/10/2025 21:10:00</c:v>
-                </c:pt>
-                <c:pt idx="128">
-                  <c:v>02/10/2025 21:20:00</c:v>
-                </c:pt>
-                <c:pt idx="129">
-                  <c:v>02/10/2025 21:30:00</c:v>
-                </c:pt>
-                <c:pt idx="130">
-                  <c:v>02/10/2025 21:40:00</c:v>
-                </c:pt>
-                <c:pt idx="131">
-                  <c:v>02/10/2025 21:50:00</c:v>
-                </c:pt>
-                <c:pt idx="132">
-                  <c:v>02/10/2025 22:00:00</c:v>
-                </c:pt>
-                <c:pt idx="133">
-                  <c:v>02/10/2025 22:10:00</c:v>
-                </c:pt>
-                <c:pt idx="134">
-                  <c:v>02/10/2025 22:20:00</c:v>
-                </c:pt>
-                <c:pt idx="135">
-                  <c:v>02/10/2025 22:30:00</c:v>
-                </c:pt>
-                <c:pt idx="136">
-                  <c:v>02/10/2025 22:40:00</c:v>
-                </c:pt>
-                <c:pt idx="137">
-                  <c:v>02/10/2025 22:50:00</c:v>
-                </c:pt>
-                <c:pt idx="138">
-                  <c:v>02/10/2025 23:00:00</c:v>
-                </c:pt>
-                <c:pt idx="139">
-                  <c:v>02/10/2025 23:10:00</c:v>
-                </c:pt>
-                <c:pt idx="140">
-                  <c:v>02/10/2025 23:20:00</c:v>
-                </c:pt>
-                <c:pt idx="141">
-                  <c:v>02/10/2025 23:30:00</c:v>
-                </c:pt>
-                <c:pt idx="142">
-                  <c:v>02/10/2025 23:40:00</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet0!$B$145:$B$287</c:f>
-              <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="143"/>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-19E1-48C8-A7C8-7210880D5D7F}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet0!$A$145:$A$287</c:f>
-              <c:strCache>
-                <c:ptCount val="143"/>
-                <c:pt idx="0">
-                  <c:v>02/10/2025 00:00:00</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>02/10/2025 00:10:00</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>02/10/2025 00:20:00</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>02/10/2025 00:30:00</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>02/10/2025 00:40:00</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>02/10/2025 00:50:00</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>02/10/2025 01:00:00</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>02/10/2025 01:10:00</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>02/10/2025 01:20:00</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>02/10/2025 01:30:00</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>02/10/2025 01:40:00</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>02/10/2025 01:50:00</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>02/10/2025 02:00:00</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>02/10/2025 02:10:00</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>02/10/2025 02:20:00</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>02/10/2025 02:30:00</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>02/10/2025 02:40:00</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>02/10/2025 02:50:00</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>02/10/2025 03:00:00</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>02/10/2025 03:10:00</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>02/10/2025 03:20:00</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>02/10/2025 03:30:00</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>02/10/2025 03:40:00</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>02/10/2025 03:50:00</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>02/10/2025 04:00:00</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>02/10/2025 04:10:00</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>02/10/2025 04:20:00</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>02/10/2025 04:30:00</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>02/10/2025 04:40:00</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>02/10/2025 04:50:00</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>02/10/2025 05:00:00</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>02/10/2025 05:10:00</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>02/10/2025 05:20:00</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>02/10/2025 05:30:00</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>02/10/2025 05:40:00</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>02/10/2025 05:50:00</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>02/10/2025 06:00:00</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>02/10/2025 06:10:00</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>02/10/2025 06:20:00</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>02/10/2025 06:30:00</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>02/10/2025 06:40:00</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>02/10/2025 06:50:00</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>02/10/2025 07:00:00</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>02/10/2025 07:10:00</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>02/10/2025 07:20:00</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>02/10/2025 07:30:00</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>02/10/2025 07:40:00</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>02/10/2025 07:50:00</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>02/10/2025 08:00:00</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>02/10/2025 08:10:00</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>02/10/2025 08:20:00</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>02/10/2025 08:30:00</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>02/10/2025 08:40:00</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>02/10/2025 08:50:00</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>02/10/2025 09:00:00</c:v>
-                </c:pt>
-                <c:pt idx="55">
-                  <c:v>02/10/2025 09:10:00</c:v>
-                </c:pt>
-                <c:pt idx="56">
-                  <c:v>02/10/2025 09:20:00</c:v>
-                </c:pt>
-                <c:pt idx="57">
-                  <c:v>02/10/2025 09:30:00</c:v>
-                </c:pt>
-                <c:pt idx="58">
-                  <c:v>02/10/2025 09:40:00</c:v>
-                </c:pt>
-                <c:pt idx="59">
-                  <c:v>02/10/2025 09:50:00</c:v>
-                </c:pt>
-                <c:pt idx="60">
-                  <c:v>02/10/2025 10:00:00</c:v>
-                </c:pt>
-                <c:pt idx="61">
-                  <c:v>02/10/2025 10:10:00</c:v>
-                </c:pt>
-                <c:pt idx="62">
-                  <c:v>02/10/2025 10:20:00</c:v>
-                </c:pt>
-                <c:pt idx="63">
-                  <c:v>02/10/2025 10:30:00</c:v>
-                </c:pt>
-                <c:pt idx="64">
-                  <c:v>02/10/2025 10:40:00</c:v>
-                </c:pt>
-                <c:pt idx="65">
-                  <c:v>02/10/2025 10:50:00</c:v>
-                </c:pt>
-                <c:pt idx="66">
-                  <c:v>02/10/2025 11:00:00</c:v>
-                </c:pt>
-                <c:pt idx="67">
-                  <c:v>02/10/2025 11:10:00</c:v>
-                </c:pt>
-                <c:pt idx="68">
-                  <c:v>02/10/2025 11:20:00</c:v>
-                </c:pt>
-                <c:pt idx="69">
-                  <c:v>02/10/2025 11:30:00</c:v>
-                </c:pt>
-                <c:pt idx="70">
-                  <c:v>02/10/2025 11:40:00</c:v>
-                </c:pt>
-                <c:pt idx="71">
-                  <c:v>02/10/2025 11:50:00</c:v>
-                </c:pt>
-                <c:pt idx="72">
-                  <c:v>02/10/2025 12:00:00</c:v>
-                </c:pt>
-                <c:pt idx="73">
-                  <c:v>02/10/2025 12:10:00</c:v>
-                </c:pt>
-                <c:pt idx="74">
-                  <c:v>02/10/2025 12:20:00</c:v>
-                </c:pt>
-                <c:pt idx="75">
-                  <c:v>02/10/2025 12:30:00</c:v>
-                </c:pt>
-                <c:pt idx="76">
-                  <c:v>02/10/2025 12:40:00</c:v>
-                </c:pt>
-                <c:pt idx="77">
-                  <c:v>02/10/2025 12:50:00</c:v>
-                </c:pt>
-                <c:pt idx="78">
-                  <c:v>02/10/2025 13:00:00</c:v>
-                </c:pt>
-                <c:pt idx="79">
-                  <c:v>02/10/2025 13:10:00</c:v>
-                </c:pt>
-                <c:pt idx="80">
-                  <c:v>02/10/2025 13:20:00</c:v>
-                </c:pt>
-                <c:pt idx="81">
-                  <c:v>02/10/2025 13:30:00</c:v>
-                </c:pt>
-                <c:pt idx="82">
-                  <c:v>02/10/2025 13:40:00</c:v>
-                </c:pt>
-                <c:pt idx="83">
-                  <c:v>02/10/2025 13:50:00</c:v>
-                </c:pt>
-                <c:pt idx="84">
-                  <c:v>02/10/2025 14:00:00</c:v>
-                </c:pt>
-                <c:pt idx="85">
-                  <c:v>02/10/2025 14:10:00</c:v>
-                </c:pt>
-                <c:pt idx="86">
-                  <c:v>02/10/2025 14:20:00</c:v>
-                </c:pt>
-                <c:pt idx="87">
-                  <c:v>02/10/2025 14:30:00</c:v>
-                </c:pt>
-                <c:pt idx="88">
-                  <c:v>02/10/2025 14:40:00</c:v>
-                </c:pt>
-                <c:pt idx="89">
-                  <c:v>02/10/2025 14:50:00</c:v>
-                </c:pt>
-                <c:pt idx="90">
-                  <c:v>02/10/2025 15:00:00</c:v>
-                </c:pt>
-                <c:pt idx="91">
-                  <c:v>02/10/2025 15:10:00</c:v>
-                </c:pt>
-                <c:pt idx="92">
-                  <c:v>02/10/2025 15:20:00</c:v>
-                </c:pt>
-                <c:pt idx="93">
-                  <c:v>02/10/2025 15:30:00</c:v>
-                </c:pt>
-                <c:pt idx="94">
-                  <c:v>02/10/2025 15:40:00</c:v>
-                </c:pt>
-                <c:pt idx="95">
-                  <c:v>02/10/2025 15:50:00</c:v>
-                </c:pt>
-                <c:pt idx="96">
-                  <c:v>02/10/2025 16:00:00</c:v>
-                </c:pt>
-                <c:pt idx="97">
-                  <c:v>02/10/2025 16:10:00</c:v>
-                </c:pt>
-                <c:pt idx="98">
-                  <c:v>02/10/2025 16:20:00</c:v>
-                </c:pt>
-                <c:pt idx="99">
-                  <c:v>02/10/2025 16:30:00</c:v>
-                </c:pt>
-                <c:pt idx="100">
-                  <c:v>02/10/2025 16:40:00</c:v>
-                </c:pt>
-                <c:pt idx="101">
-                  <c:v>02/10/2025 16:50:00</c:v>
-                </c:pt>
-                <c:pt idx="102">
-                  <c:v>02/10/2025 17:00:00</c:v>
-                </c:pt>
-                <c:pt idx="103">
-                  <c:v>02/10/2025 17:10:00</c:v>
-                </c:pt>
-                <c:pt idx="104">
-                  <c:v>02/10/2025 17:20:00</c:v>
-                </c:pt>
-                <c:pt idx="105">
-                  <c:v>02/10/2025 17:30:00</c:v>
-                </c:pt>
-                <c:pt idx="106">
-                  <c:v>02/10/2025 17:40:00</c:v>
-                </c:pt>
-                <c:pt idx="107">
-                  <c:v>02/10/2025 17:50:00</c:v>
-                </c:pt>
-                <c:pt idx="108">
-                  <c:v>02/10/2025 18:00:00</c:v>
-                </c:pt>
-                <c:pt idx="109">
-                  <c:v>02/10/2025 18:10:00</c:v>
-                </c:pt>
-                <c:pt idx="110">
-                  <c:v>02/10/2025 18:20:00</c:v>
-                </c:pt>
-                <c:pt idx="111">
-                  <c:v>02/10/2025 18:30:00</c:v>
-                </c:pt>
-                <c:pt idx="112">
-                  <c:v>02/10/2025 18:40:00</c:v>
-                </c:pt>
-                <c:pt idx="113">
-                  <c:v>02/10/2025 18:50:00</c:v>
-                </c:pt>
-                <c:pt idx="114">
-                  <c:v>02/10/2025 19:00:00</c:v>
-                </c:pt>
-                <c:pt idx="115">
-                  <c:v>02/10/2025 19:10:00</c:v>
-                </c:pt>
-                <c:pt idx="116">
-                  <c:v>02/10/2025 19:20:00</c:v>
-                </c:pt>
-                <c:pt idx="117">
-                  <c:v>02/10/2025 19:30:00</c:v>
-                </c:pt>
-                <c:pt idx="118">
-                  <c:v>02/10/2025 19:40:00</c:v>
-                </c:pt>
-                <c:pt idx="119">
-                  <c:v>02/10/2025 19:50:00</c:v>
-                </c:pt>
-                <c:pt idx="120">
-                  <c:v>02/10/2025 20:00:00</c:v>
-                </c:pt>
-                <c:pt idx="121">
-                  <c:v>02/10/2025 20:10:00</c:v>
-                </c:pt>
-                <c:pt idx="122">
-                  <c:v>02/10/2025 20:20:00</c:v>
-                </c:pt>
-                <c:pt idx="123">
-                  <c:v>02/10/2025 20:30:00</c:v>
-                </c:pt>
-                <c:pt idx="124">
-                  <c:v>02/10/2025 20:40:00</c:v>
-                </c:pt>
-                <c:pt idx="125">
-                  <c:v>02/10/2025 20:50:00</c:v>
-                </c:pt>
-                <c:pt idx="126">
-                  <c:v>02/10/2025 21:00:00</c:v>
-                </c:pt>
-                <c:pt idx="127">
-                  <c:v>02/10/2025 21:10:00</c:v>
-                </c:pt>
-                <c:pt idx="128">
-                  <c:v>02/10/2025 21:20:00</c:v>
-                </c:pt>
-                <c:pt idx="129">
-                  <c:v>02/10/2025 21:30:00</c:v>
-                </c:pt>
-                <c:pt idx="130">
-                  <c:v>02/10/2025 21:40:00</c:v>
-                </c:pt>
-                <c:pt idx="131">
-                  <c:v>02/10/2025 21:50:00</c:v>
-                </c:pt>
-                <c:pt idx="132">
-                  <c:v>02/10/2025 22:00:00</c:v>
-                </c:pt>
-                <c:pt idx="133">
-                  <c:v>02/10/2025 22:10:00</c:v>
-                </c:pt>
-                <c:pt idx="134">
-                  <c:v>02/10/2025 22:20:00</c:v>
-                </c:pt>
-                <c:pt idx="135">
-                  <c:v>02/10/2025 22:30:00</c:v>
-                </c:pt>
-                <c:pt idx="136">
-                  <c:v>02/10/2025 22:40:00</c:v>
-                </c:pt>
-                <c:pt idx="137">
-                  <c:v>02/10/2025 22:50:00</c:v>
-                </c:pt>
-                <c:pt idx="138">
-                  <c:v>02/10/2025 23:00:00</c:v>
-                </c:pt>
-                <c:pt idx="139">
-                  <c:v>02/10/2025 23:10:00</c:v>
-                </c:pt>
-                <c:pt idx="140">
-                  <c:v>02/10/2025 23:20:00</c:v>
-                </c:pt>
-                <c:pt idx="141">
-                  <c:v>02/10/2025 23:30:00</c:v>
-                </c:pt>
-                <c:pt idx="142">
-                  <c:v>02/10/2025 23:40:00</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet0!$C$145:$C$287</c:f>
-              <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="143"/>
-                <c:pt idx="0">
-                  <c:v>28.338462829589844</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>28.288457870483398</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>28.238458633422852</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>28.215381622314453</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>28.165382385253906</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>28.092306137084961</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>28.065383911132813</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>27.992307662963867</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>27.94230842590332</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>27.892309188842773</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>27.842309951782227</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>27.792304992675781</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>28.319229125976563</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>34.911537170410156</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>41.534614562988281</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>48.126922607421875</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>53.700000762939453</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>59.273075103759766</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>64.976921081542969</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>71.699996948242188</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>78.376914978027344</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>84.403839111328125</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>84.380760192871094</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>84.380760192871094</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>84.27691650390625</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>84.25384521484375</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>84.203842163085938</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>84.180763244628906</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>84.103843688964844</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>84.080764770507813</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>84.00384521484375</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>83.953849792480469</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>83.953849792480469</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>83.853843688964844</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>83.853843688964844</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>83.803840637207031</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>83.730758666992188</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>83.707695007324219</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>83.657699584960938</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>83.584617614746094</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>83.53460693359375</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>83.484603881835938</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>82.76153564453125</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>74.78460693359375</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>66.907691955566406</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>58.857692718505859</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>46.153842926025391</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>33.526920318603516</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>21.830766677856445</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>21.80769157409668</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>21.784616470336914</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>21.734613418579102</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>21.707691192626953</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>21.661537170410156</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>21.426923751831055</c:v>
-                </c:pt>
-                <c:pt idx="55">
-                  <c:v>20.176921844482422</c:v>
-                </c:pt>
-                <c:pt idx="56">
-                  <c:v>20.034614562988281</c:v>
-                </c:pt>
-                <c:pt idx="57">
-                  <c:v>19.880767822265625</c:v>
-                </c:pt>
-                <c:pt idx="58">
-                  <c:v>19.788459777832031</c:v>
-                </c:pt>
-                <c:pt idx="59">
-                  <c:v>19.473075866699219</c:v>
-                </c:pt>
-                <c:pt idx="60">
-                  <c:v>19.31153678894043</c:v>
-                </c:pt>
-                <c:pt idx="61">
-                  <c:v>19.165382385253906</c:v>
-                </c:pt>
-                <c:pt idx="62">
-                  <c:v>19.069229125976563</c:v>
-                </c:pt>
-                <c:pt idx="63">
-                  <c:v>19.069229125976563</c:v>
-                </c:pt>
-                <c:pt idx="64">
-                  <c:v>18.899997711181641</c:v>
-                </c:pt>
-                <c:pt idx="65">
-                  <c:v>18.780769348144531</c:v>
-                </c:pt>
-                <c:pt idx="66">
-                  <c:v>18.623075485229492</c:v>
-                </c:pt>
-                <c:pt idx="67">
-                  <c:v>18.242305755615234</c:v>
-                </c:pt>
-                <c:pt idx="68">
-                  <c:v>18.142307281494141</c:v>
-                </c:pt>
-                <c:pt idx="69">
-                  <c:v>18.088462829589844</c:v>
-                </c:pt>
-                <c:pt idx="70">
-                  <c:v>17.942306518554688</c:v>
-                </c:pt>
-                <c:pt idx="71">
-                  <c:v>17.873075485229492</c:v>
-                </c:pt>
-                <c:pt idx="72">
-                  <c:v>17.846153259277344</c:v>
-                </c:pt>
-                <c:pt idx="73">
-                  <c:v>17.750001907348633</c:v>
-                </c:pt>
-                <c:pt idx="74">
-                  <c:v>17.746152877807617</c:v>
-                </c:pt>
-                <c:pt idx="75">
-                  <c:v>17.623077392578125</c:v>
-                </c:pt>
-                <c:pt idx="76">
-                  <c:v>17.526922225952148</c:v>
-                </c:pt>
-                <c:pt idx="77">
-                  <c:v>17.500001907348633</c:v>
-                </c:pt>
-                <c:pt idx="78">
-                  <c:v>17.642309188842773</c:v>
-                </c:pt>
-                <c:pt idx="79">
-                  <c:v>21.669229507446289</c:v>
-                </c:pt>
-                <c:pt idx="80">
-                  <c:v>25.692306518554688</c:v>
-                </c:pt>
-                <c:pt idx="81">
-                  <c:v>29.865385055541992</c:v>
-                </c:pt>
-                <c:pt idx="82">
-                  <c:v>36.461540222167969</c:v>
-                </c:pt>
-                <c:pt idx="83">
-                  <c:v>43.180770874023438</c:v>
-                </c:pt>
-                <c:pt idx="84">
-                  <c:v>49.907688140869141</c:v>
-                </c:pt>
-                <c:pt idx="85">
-                  <c:v>56.607696533203125</c:v>
-                </c:pt>
-                <c:pt idx="86">
-                  <c:v>63.330764770507813</c:v>
-                </c:pt>
-                <c:pt idx="87">
-                  <c:v>70.157691955566406</c:v>
-                </c:pt>
-                <c:pt idx="88">
-                  <c:v>76.880767822265625</c:v>
-                </c:pt>
-                <c:pt idx="89">
-                  <c:v>83.630760192871094</c:v>
-                </c:pt>
-                <c:pt idx="90">
-                  <c:v>89.634613037109375</c:v>
-                </c:pt>
-                <c:pt idx="91">
-                  <c:v>89.584609985351563</c:v>
-                </c:pt>
-                <c:pt idx="92">
-                  <c:v>89.534614562988281</c:v>
-                </c:pt>
-                <c:pt idx="93">
-                  <c:v>89.484611511230469</c:v>
-                </c:pt>
-                <c:pt idx="94">
-                  <c:v>89.407699584960938</c:v>
-                </c:pt>
-                <c:pt idx="95">
-                  <c:v>89.384613037109375</c:v>
-                </c:pt>
-                <c:pt idx="96">
-                  <c:v>89.357688903808594</c:v>
-                </c:pt>
-                <c:pt idx="97">
-                  <c:v>89.284614562988281</c:v>
-                </c:pt>
-                <c:pt idx="98">
-                  <c:v>89.284614562988281</c:v>
-                </c:pt>
-                <c:pt idx="99">
-                  <c:v>89.184608459472656</c:v>
-                </c:pt>
-                <c:pt idx="100">
-                  <c:v>89.184608459472656</c:v>
-                </c:pt>
-                <c:pt idx="101">
-                  <c:v>89.134613037109375</c:v>
-                </c:pt>
-                <c:pt idx="102">
-                  <c:v>89.084617614746094</c:v>
-                </c:pt>
-                <c:pt idx="103">
-                  <c:v>89.057693481445313</c:v>
-                </c:pt>
-                <c:pt idx="104">
-                  <c:v>88.984619140625</c:v>
-                </c:pt>
-                <c:pt idx="105">
-                  <c:v>88.957687377929688</c:v>
-                </c:pt>
-                <c:pt idx="106">
-                  <c:v>88.911537170410156</c:v>
-                </c:pt>
-                <c:pt idx="107">
-                  <c:v>88.857688903808594</c:v>
-                </c:pt>
-                <c:pt idx="108">
-                  <c:v>87.561531066894531</c:v>
-                </c:pt>
-                <c:pt idx="109">
-                  <c:v>74.084617614746094</c:v>
-                </c:pt>
-                <c:pt idx="110">
-                  <c:v>61.184612274169922</c:v>
-                </c:pt>
-                <c:pt idx="111">
-                  <c:v>48.930763244628906</c:v>
-                </c:pt>
-                <c:pt idx="112">
-                  <c:v>42.184612274169922</c:v>
-                </c:pt>
-                <c:pt idx="113">
-                  <c:v>35.411537170410156</c:v>
-                </c:pt>
-                <c:pt idx="114">
-                  <c:v>29.184616088867188</c:v>
-                </c:pt>
-                <c:pt idx="115">
-                  <c:v>29.107688903808594</c:v>
-                </c:pt>
-                <c:pt idx="116">
-                  <c:v>29.107688903808594</c:v>
-                </c:pt>
-                <c:pt idx="117">
-                  <c:v>29.084615707397461</c:v>
-                </c:pt>
-                <c:pt idx="118">
-                  <c:v>29.057689666748047</c:v>
-                </c:pt>
-                <c:pt idx="119">
-                  <c:v>29.0076904296875</c:v>
-                </c:pt>
-                <c:pt idx="120">
-                  <c:v>28.930768966674805</c:v>
-                </c:pt>
-                <c:pt idx="121">
-                  <c:v>28.907691955566406</c:v>
-                </c:pt>
-                <c:pt idx="122">
-                  <c:v>28.830766677856445</c:v>
-                </c:pt>
-                <c:pt idx="123">
-                  <c:v>28.780767440795898</c:v>
-                </c:pt>
-                <c:pt idx="124">
-                  <c:v>28.707691192626953</c:v>
-                </c:pt>
-                <c:pt idx="125">
-                  <c:v>28.657690048217773</c:v>
-                </c:pt>
-                <c:pt idx="126">
-                  <c:v>28.607690811157227</c:v>
-                </c:pt>
-                <c:pt idx="127">
-                  <c:v>28.5076904296875</c:v>
-                </c:pt>
-                <c:pt idx="128">
-                  <c:v>28.480768203735352</c:v>
-                </c:pt>
-                <c:pt idx="129">
-                  <c:v>28.407691955566406</c:v>
-                </c:pt>
-                <c:pt idx="130">
-                  <c:v>28.357690811157227</c:v>
-                </c:pt>
-                <c:pt idx="131">
-                  <c:v>28.280765533447266</c:v>
-                </c:pt>
-                <c:pt idx="132">
-                  <c:v>28.207691192626953</c:v>
-                </c:pt>
-                <c:pt idx="133">
-                  <c:v>28.180768966674805</c:v>
-                </c:pt>
-                <c:pt idx="134">
-                  <c:v>28.107690811157227</c:v>
-                </c:pt>
-                <c:pt idx="135">
-                  <c:v>28.307689666748047</c:v>
-                </c:pt>
-                <c:pt idx="136">
-                  <c:v>31.234613418579102</c:v>
-                </c:pt>
-                <c:pt idx="137">
-                  <c:v>34.207695007324219</c:v>
-                </c:pt>
-                <c:pt idx="138">
-                  <c:v>36.830772399902344</c:v>
-                </c:pt>
-                <c:pt idx="139">
-                  <c:v>36.753841400146484</c:v>
-                </c:pt>
-                <c:pt idx="140">
-                  <c:v>36.730766296386719</c:v>
-                </c:pt>
-                <c:pt idx="141">
-                  <c:v>36.653846740722656</c:v>
-                </c:pt>
-                <c:pt idx="142">
-                  <c:v>36.607688903808594</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-19E1-48C8-A7C8-7210880D5D7F}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet0!$A$145:$A$287</c:f>
-              <c:strCache>
-                <c:ptCount val="143"/>
-                <c:pt idx="0">
-                  <c:v>02/10/2025 00:00:00</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>02/10/2025 00:10:00</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>02/10/2025 00:20:00</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>02/10/2025 00:30:00</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>02/10/2025 00:40:00</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>02/10/2025 00:50:00</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>02/10/2025 01:00:00</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>02/10/2025 01:10:00</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>02/10/2025 01:20:00</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>02/10/2025 01:30:00</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>02/10/2025 01:40:00</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>02/10/2025 01:50:00</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>02/10/2025 02:00:00</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>02/10/2025 02:10:00</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>02/10/2025 02:20:00</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>02/10/2025 02:30:00</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>02/10/2025 02:40:00</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>02/10/2025 02:50:00</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>02/10/2025 03:00:00</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>02/10/2025 03:10:00</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>02/10/2025 03:20:00</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>02/10/2025 03:30:00</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>02/10/2025 03:40:00</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>02/10/2025 03:50:00</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>02/10/2025 04:00:00</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>02/10/2025 04:10:00</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>02/10/2025 04:20:00</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>02/10/2025 04:30:00</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>02/10/2025 04:40:00</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>02/10/2025 04:50:00</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>02/10/2025 05:00:00</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>02/10/2025 05:10:00</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>02/10/2025 05:20:00</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>02/10/2025 05:30:00</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>02/10/2025 05:40:00</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>02/10/2025 05:50:00</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>02/10/2025 06:00:00</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>02/10/2025 06:10:00</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>02/10/2025 06:20:00</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>02/10/2025 06:30:00</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>02/10/2025 06:40:00</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>02/10/2025 06:50:00</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>02/10/2025 07:00:00</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>02/10/2025 07:10:00</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>02/10/2025 07:20:00</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>02/10/2025 07:30:00</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>02/10/2025 07:40:00</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>02/10/2025 07:50:00</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>02/10/2025 08:00:00</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>02/10/2025 08:10:00</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>02/10/2025 08:20:00</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>02/10/2025 08:30:00</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>02/10/2025 08:40:00</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>02/10/2025 08:50:00</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>02/10/2025 09:00:00</c:v>
-                </c:pt>
-                <c:pt idx="55">
-                  <c:v>02/10/2025 09:10:00</c:v>
-                </c:pt>
-                <c:pt idx="56">
-                  <c:v>02/10/2025 09:20:00</c:v>
-                </c:pt>
-                <c:pt idx="57">
-                  <c:v>02/10/2025 09:30:00</c:v>
-                </c:pt>
-                <c:pt idx="58">
-                  <c:v>02/10/2025 09:40:00</c:v>
-                </c:pt>
-                <c:pt idx="59">
-                  <c:v>02/10/2025 09:50:00</c:v>
-                </c:pt>
-                <c:pt idx="60">
-                  <c:v>02/10/2025 10:00:00</c:v>
-                </c:pt>
-                <c:pt idx="61">
-                  <c:v>02/10/2025 10:10:00</c:v>
-                </c:pt>
-                <c:pt idx="62">
-                  <c:v>02/10/2025 10:20:00</c:v>
-                </c:pt>
-                <c:pt idx="63">
-                  <c:v>02/10/2025 10:30:00</c:v>
-                </c:pt>
-                <c:pt idx="64">
-                  <c:v>02/10/2025 10:40:00</c:v>
-                </c:pt>
-                <c:pt idx="65">
-                  <c:v>02/10/2025 10:50:00</c:v>
-                </c:pt>
-                <c:pt idx="66">
-                  <c:v>02/10/2025 11:00:00</c:v>
-                </c:pt>
-                <c:pt idx="67">
-                  <c:v>02/10/2025 11:10:00</c:v>
-                </c:pt>
-                <c:pt idx="68">
-                  <c:v>02/10/2025 11:20:00</c:v>
-                </c:pt>
-                <c:pt idx="69">
-                  <c:v>02/10/2025 11:30:00</c:v>
-                </c:pt>
-                <c:pt idx="70">
-                  <c:v>02/10/2025 11:40:00</c:v>
-                </c:pt>
-                <c:pt idx="71">
-                  <c:v>02/10/2025 11:50:00</c:v>
-                </c:pt>
-                <c:pt idx="72">
-                  <c:v>02/10/2025 12:00:00</c:v>
-                </c:pt>
-                <c:pt idx="73">
-                  <c:v>02/10/2025 12:10:00</c:v>
-                </c:pt>
-                <c:pt idx="74">
-                  <c:v>02/10/2025 12:20:00</c:v>
-                </c:pt>
-                <c:pt idx="75">
-                  <c:v>02/10/2025 12:30:00</c:v>
-                </c:pt>
-                <c:pt idx="76">
-                  <c:v>02/10/2025 12:40:00</c:v>
-                </c:pt>
-                <c:pt idx="77">
-                  <c:v>02/10/2025 12:50:00</c:v>
-                </c:pt>
-                <c:pt idx="78">
-                  <c:v>02/10/2025 13:00:00</c:v>
-                </c:pt>
-                <c:pt idx="79">
-                  <c:v>02/10/2025 13:10:00</c:v>
-                </c:pt>
-                <c:pt idx="80">
-                  <c:v>02/10/2025 13:20:00</c:v>
-                </c:pt>
-                <c:pt idx="81">
-                  <c:v>02/10/2025 13:30:00</c:v>
-                </c:pt>
-                <c:pt idx="82">
-                  <c:v>02/10/2025 13:40:00</c:v>
-                </c:pt>
-                <c:pt idx="83">
-                  <c:v>02/10/2025 13:50:00</c:v>
-                </c:pt>
-                <c:pt idx="84">
-                  <c:v>02/10/2025 14:00:00</c:v>
-                </c:pt>
-                <c:pt idx="85">
-                  <c:v>02/10/2025 14:10:00</c:v>
-                </c:pt>
-                <c:pt idx="86">
-                  <c:v>02/10/2025 14:20:00</c:v>
-                </c:pt>
-                <c:pt idx="87">
-                  <c:v>02/10/2025 14:30:00</c:v>
-                </c:pt>
-                <c:pt idx="88">
-                  <c:v>02/10/2025 14:40:00</c:v>
-                </c:pt>
-                <c:pt idx="89">
-                  <c:v>02/10/2025 14:50:00</c:v>
-                </c:pt>
-                <c:pt idx="90">
-                  <c:v>02/10/2025 15:00:00</c:v>
-                </c:pt>
-                <c:pt idx="91">
-                  <c:v>02/10/2025 15:10:00</c:v>
-                </c:pt>
-                <c:pt idx="92">
-                  <c:v>02/10/2025 15:20:00</c:v>
-                </c:pt>
-                <c:pt idx="93">
-                  <c:v>02/10/2025 15:30:00</c:v>
-                </c:pt>
-                <c:pt idx="94">
-                  <c:v>02/10/2025 15:40:00</c:v>
-                </c:pt>
-                <c:pt idx="95">
-                  <c:v>02/10/2025 15:50:00</c:v>
-                </c:pt>
-                <c:pt idx="96">
-                  <c:v>02/10/2025 16:00:00</c:v>
-                </c:pt>
-                <c:pt idx="97">
-                  <c:v>02/10/2025 16:10:00</c:v>
-                </c:pt>
-                <c:pt idx="98">
-                  <c:v>02/10/2025 16:20:00</c:v>
-                </c:pt>
-                <c:pt idx="99">
-                  <c:v>02/10/2025 16:30:00</c:v>
-                </c:pt>
-                <c:pt idx="100">
-                  <c:v>02/10/2025 16:40:00</c:v>
-                </c:pt>
-                <c:pt idx="101">
-                  <c:v>02/10/2025 16:50:00</c:v>
-                </c:pt>
-                <c:pt idx="102">
-                  <c:v>02/10/2025 17:00:00</c:v>
-                </c:pt>
-                <c:pt idx="103">
-                  <c:v>02/10/2025 17:10:00</c:v>
-                </c:pt>
-                <c:pt idx="104">
-                  <c:v>02/10/2025 17:20:00</c:v>
-                </c:pt>
-                <c:pt idx="105">
-                  <c:v>02/10/2025 17:30:00</c:v>
-                </c:pt>
-                <c:pt idx="106">
-                  <c:v>02/10/2025 17:40:00</c:v>
-                </c:pt>
-                <c:pt idx="107">
-                  <c:v>02/10/2025 17:50:00</c:v>
-                </c:pt>
-                <c:pt idx="108">
-                  <c:v>02/10/2025 18:00:00</c:v>
-                </c:pt>
-                <c:pt idx="109">
-                  <c:v>02/10/2025 18:10:00</c:v>
-                </c:pt>
-                <c:pt idx="110">
-                  <c:v>02/10/2025 18:20:00</c:v>
-                </c:pt>
-                <c:pt idx="111">
-                  <c:v>02/10/2025 18:30:00</c:v>
-                </c:pt>
-                <c:pt idx="112">
-                  <c:v>02/10/2025 18:40:00</c:v>
-                </c:pt>
-                <c:pt idx="113">
-                  <c:v>02/10/2025 18:50:00</c:v>
-                </c:pt>
-                <c:pt idx="114">
-                  <c:v>02/10/2025 19:00:00</c:v>
-                </c:pt>
-                <c:pt idx="115">
-                  <c:v>02/10/2025 19:10:00</c:v>
-                </c:pt>
-                <c:pt idx="116">
-                  <c:v>02/10/2025 19:20:00</c:v>
-                </c:pt>
-                <c:pt idx="117">
-                  <c:v>02/10/2025 19:30:00</c:v>
-                </c:pt>
-                <c:pt idx="118">
-                  <c:v>02/10/2025 19:40:00</c:v>
-                </c:pt>
-                <c:pt idx="119">
-                  <c:v>02/10/2025 19:50:00</c:v>
-                </c:pt>
-                <c:pt idx="120">
-                  <c:v>02/10/2025 20:00:00</c:v>
-                </c:pt>
-                <c:pt idx="121">
-                  <c:v>02/10/2025 20:10:00</c:v>
-                </c:pt>
-                <c:pt idx="122">
-                  <c:v>02/10/2025 20:20:00</c:v>
-                </c:pt>
-                <c:pt idx="123">
-                  <c:v>02/10/2025 20:30:00</c:v>
-                </c:pt>
-                <c:pt idx="124">
-                  <c:v>02/10/2025 20:40:00</c:v>
-                </c:pt>
-                <c:pt idx="125">
-                  <c:v>02/10/2025 20:50:00</c:v>
-                </c:pt>
-                <c:pt idx="126">
-                  <c:v>02/10/2025 21:00:00</c:v>
-                </c:pt>
-                <c:pt idx="127">
-                  <c:v>02/10/2025 21:10:00</c:v>
-                </c:pt>
-                <c:pt idx="128">
-                  <c:v>02/10/2025 21:20:00</c:v>
-                </c:pt>
-                <c:pt idx="129">
-                  <c:v>02/10/2025 21:30:00</c:v>
-                </c:pt>
-                <c:pt idx="130">
-                  <c:v>02/10/2025 21:40:00</c:v>
-                </c:pt>
-                <c:pt idx="131">
-                  <c:v>02/10/2025 21:50:00</c:v>
-                </c:pt>
-                <c:pt idx="132">
-                  <c:v>02/10/2025 22:00:00</c:v>
-                </c:pt>
-                <c:pt idx="133">
-                  <c:v>02/10/2025 22:10:00</c:v>
-                </c:pt>
-                <c:pt idx="134">
-                  <c:v>02/10/2025 22:20:00</c:v>
-                </c:pt>
-                <c:pt idx="135">
-                  <c:v>02/10/2025 22:30:00</c:v>
-                </c:pt>
-                <c:pt idx="136">
-                  <c:v>02/10/2025 22:40:00</c:v>
-                </c:pt>
-                <c:pt idx="137">
-                  <c:v>02/10/2025 22:50:00</c:v>
-                </c:pt>
-                <c:pt idx="138">
-                  <c:v>02/10/2025 23:00:00</c:v>
-                </c:pt>
-                <c:pt idx="139">
-                  <c:v>02/10/2025 23:10:00</c:v>
-                </c:pt>
-                <c:pt idx="140">
-                  <c:v>02/10/2025 23:20:00</c:v>
-                </c:pt>
-                <c:pt idx="141">
-                  <c:v>02/10/2025 23:30:00</c:v>
-                </c:pt>
-                <c:pt idx="142">
-                  <c:v>02/10/2025 23:40:00</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet0!$D$145:$D$287</c:f>
-              <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="143"/>
-                <c:pt idx="0">
-                  <c:v>1.6051026582717896</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1.6188194751739502</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1.4700981378555298</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1.6400631666183472</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1.6394722461700439</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1.6185257434844971</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>1.5916227102279663</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1.7093774080276489</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.7081996202468872</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1.661371111869812</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>1.7187718152999878</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>1.6410782337188721</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>-362.56988525390625</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>-3984.49560546875</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>-3984.5927734375</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>-3909.871337890625</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>-3299.06982421875</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>-3299.04248046875</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>-3363.05029296875</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>-3966.04931640625</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>-3966.1328125</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>-3597.561767578125</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>1.2782179117202759</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>1.6917227506637573</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>1.6123433113098145</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>1.6251736879348755</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>1.5712337493896484</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>1.6403858661651611</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>1.5164808034896851</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>1.5496507883071899</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>0.89734143018722534</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>1.4545613527297974</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>1.4916070699691772</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>1.6633323431015015</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>1.673799991607666</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>1.5694938898086548</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>1.0980079174041748</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>1.6521021127700806</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>1.5257472991943359</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>1.4296859502792358</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>1.4269664287567139</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>1.5241613388061523</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>406.82369995117188</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>4302.07568359375</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>4293.42529296875</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>4560.69091796875</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>7201.16015625</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>7195.86572265625</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>6550.4658203125</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>1.7096383571624756</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>1.7297621965408325</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>1.7515383958816528</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>1.8755844831466675</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>1.9291778802871704</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>1.8654190301895142</c:v>
-                </c:pt>
-                <c:pt idx="55">
-                  <c:v>1.8179183006286621</c:v>
-                </c:pt>
-                <c:pt idx="56">
-                  <c:v>1.8323084115982056</c:v>
-                </c:pt>
-                <c:pt idx="57">
-                  <c:v>1.8185365200042725</c:v>
-                </c:pt>
-                <c:pt idx="58">
-                  <c:v>1.829026460647583</c:v>
-                </c:pt>
-                <c:pt idx="59">
-                  <c:v>1.7769110202789307</c:v>
-                </c:pt>
-                <c:pt idx="60">
-                  <c:v>1.7532112598419189</c:v>
-                </c:pt>
-                <c:pt idx="61">
-                  <c:v>1.7581498622894287</c:v>
-                </c:pt>
-                <c:pt idx="62">
-                  <c:v>1.7632818222045898</c:v>
-                </c:pt>
-                <c:pt idx="63">
-                  <c:v>1.7972694635391235</c:v>
-                </c:pt>
-                <c:pt idx="64">
-                  <c:v>1.7569187879562378</c:v>
-                </c:pt>
-                <c:pt idx="65">
-                  <c:v>1.8262065649032593</c:v>
-                </c:pt>
-                <c:pt idx="66">
-                  <c:v>1.7985073328018188</c:v>
-                </c:pt>
-                <c:pt idx="67">
-                  <c:v>1.9608629941940308</c:v>
-                </c:pt>
-                <c:pt idx="68">
-                  <c:v>1.8696380853652954</c:v>
-                </c:pt>
-                <c:pt idx="69">
-                  <c:v>1.9246875047683716</c:v>
-                </c:pt>
-                <c:pt idx="70">
-                  <c:v>1.9927419424057007</c:v>
-                </c:pt>
-                <c:pt idx="71">
-                  <c:v>2.0830907821655273</c:v>
-                </c:pt>
-                <c:pt idx="72">
-                  <c:v>2.0034420490264893</c:v>
-                </c:pt>
-                <c:pt idx="73">
-                  <c:v>1.9834215641021729</c:v>
-                </c:pt>
-                <c:pt idx="74">
-                  <c:v>1.9832391738891602</c:v>
-                </c:pt>
-                <c:pt idx="75">
-                  <c:v>2.0860912799835205</c:v>
-                </c:pt>
-                <c:pt idx="76">
-                  <c:v>2.0386893749237061</c:v>
-                </c:pt>
-                <c:pt idx="77">
-                  <c:v>2.0009536743164063</c:v>
-                </c:pt>
-                <c:pt idx="78">
-                  <c:v>-221.1832275390625</c:v>
-                </c:pt>
-                <c:pt idx="79">
-                  <c:v>-2401.593017578125</c:v>
-                </c:pt>
-                <c:pt idx="80">
-                  <c:v>-2401.56591796875</c:v>
-                </c:pt>
-                <c:pt idx="81">
-                  <c:v>-2543.5478515625</c:v>
-                </c:pt>
-                <c:pt idx="82">
-                  <c:v>-3996.0908203125</c:v>
-                </c:pt>
-                <c:pt idx="83">
-                  <c:v>-3998.51904296875</c:v>
-                </c:pt>
-                <c:pt idx="84">
-                  <c:v>-3999.8955078125</c:v>
-                </c:pt>
-                <c:pt idx="85">
-                  <c:v>-4001.44287109375</c:v>
-                </c:pt>
-                <c:pt idx="86">
-                  <c:v>-3998.287841796875</c:v>
-                </c:pt>
-                <c:pt idx="87">
-                  <c:v>-4002.1103515625</c:v>
-                </c:pt>
-                <c:pt idx="88">
-                  <c:v>-4002.203369140625</c:v>
-                </c:pt>
-                <c:pt idx="89">
-                  <c:v>-3999.816162109375</c:v>
-                </c:pt>
-                <c:pt idx="90">
-                  <c:v>-3631.8271484375</c:v>
-                </c:pt>
-                <c:pt idx="91">
-                  <c:v>2.087735652923584</c:v>
-                </c:pt>
-                <c:pt idx="92">
-                  <c:v>2.0144879817962646</c:v>
-                </c:pt>
-                <c:pt idx="93">
-                  <c:v>1.9612952470779419</c:v>
-                </c:pt>
-                <c:pt idx="94">
-                  <c:v>1.910813570022583</c:v>
-                </c:pt>
-                <c:pt idx="95">
-                  <c:v>1.9918497800827026</c:v>
-                </c:pt>
-                <c:pt idx="96">
-                  <c:v>2.1007437705993652</c:v>
-                </c:pt>
-                <c:pt idx="97">
-                  <c:v>1.7802779674530029</c:v>
-                </c:pt>
-                <c:pt idx="98">
-                  <c:v>1.9510766267776489</c:v>
-                </c:pt>
-                <c:pt idx="99">
-                  <c:v>1.9355148077011108</c:v>
-                </c:pt>
-                <c:pt idx="100">
-                  <c:v>1.8729885816574097</c:v>
-                </c:pt>
-                <c:pt idx="101">
-                  <c:v>1.8231470584869385</c:v>
-                </c:pt>
-                <c:pt idx="102">
-                  <c:v>1.828880786895752</c:v>
-                </c:pt>
-                <c:pt idx="103">
-                  <c:v>1.9006986618041992</c:v>
-                </c:pt>
-                <c:pt idx="104">
-                  <c:v>1.8741739988327026</c:v>
-                </c:pt>
-                <c:pt idx="105">
-                  <c:v>1.8079468011856079</c:v>
-                </c:pt>
-                <c:pt idx="106">
-                  <c:v>1.8749512434005737</c:v>
-                </c:pt>
-                <c:pt idx="107">
-                  <c:v>1.7028336524963379</c:v>
-                </c:pt>
-                <c:pt idx="108">
-                  <c:v>690.93798828125</c:v>
-                </c:pt>
-                <c:pt idx="109">
-                  <c:v>7305.52880859375</c:v>
-                </c:pt>
-                <c:pt idx="110">
-                  <c:v>7295.9365234375</c:v>
-                </c:pt>
-                <c:pt idx="111">
-                  <c:v>6981.38671875</c:v>
-                </c:pt>
-                <c:pt idx="112">
-                  <c:v>3896.463134765625</c:v>
-                </c:pt>
-                <c:pt idx="113">
-                  <c:v>3899.344970703125</c:v>
-                </c:pt>
-                <c:pt idx="114">
-                  <c:v>3544.408935546875</c:v>
-                </c:pt>
-                <c:pt idx="115">
-                  <c:v>1.9114304780960083</c:v>
-                </c:pt>
-                <c:pt idx="116">
-                  <c:v>1.8165323734283447</c:v>
-                </c:pt>
-                <c:pt idx="117">
-                  <c:v>2.0588715076446533</c:v>
-                </c:pt>
-                <c:pt idx="118">
-                  <c:v>1.9184474945068359</c:v>
-                </c:pt>
-                <c:pt idx="119">
-                  <c:v>1.8165265321731567</c:v>
-                </c:pt>
-                <c:pt idx="120">
-                  <c:v>1.906322717666626</c:v>
-                </c:pt>
-                <c:pt idx="121">
-                  <c:v>1.8325655460357666</c:v>
-                </c:pt>
-                <c:pt idx="122">
-                  <c:v>1.7187725305557251</c:v>
-                </c:pt>
-                <c:pt idx="123">
-                  <c:v>1.9211620092391968</c:v>
-                </c:pt>
-                <c:pt idx="124">
-                  <c:v>1.7941192388534546</c:v>
-                </c:pt>
-                <c:pt idx="125">
-                  <c:v>1.9296810626983643</c:v>
-                </c:pt>
-                <c:pt idx="126">
-                  <c:v>1.97607421875</c:v>
-                </c:pt>
-                <c:pt idx="127">
-                  <c:v>1.8205163478851318</c:v>
-                </c:pt>
-                <c:pt idx="128">
-                  <c:v>1.8566223382949829</c:v>
-                </c:pt>
-                <c:pt idx="129">
-                  <c:v>1.7353620529174805</c:v>
-                </c:pt>
-                <c:pt idx="130">
-                  <c:v>1.6789671182632446</c:v>
-                </c:pt>
-                <c:pt idx="131">
-                  <c:v>1.8328665494918823</c:v>
-                </c:pt>
-                <c:pt idx="132">
-                  <c:v>1.8497238159179688</c:v>
-                </c:pt>
-                <c:pt idx="133">
-                  <c:v>1.8267172574996948</c:v>
-                </c:pt>
-                <c:pt idx="134">
-                  <c:v>1.9679819345474243</c:v>
-                </c:pt>
-                <c:pt idx="135">
-                  <c:v>-162.29782104492188</c:v>
-                </c:pt>
-                <c:pt idx="136">
-                  <c:v>-1799.9036865234375</c:v>
-                </c:pt>
-                <c:pt idx="137">
-                  <c:v>-1804.841552734375</c:v>
-                </c:pt>
-                <c:pt idx="138">
-                  <c:v>-1627.806396484375</c:v>
-                </c:pt>
-                <c:pt idx="139">
-                  <c:v>1.8951874971389771</c:v>
-                </c:pt>
-                <c:pt idx="140">
-                  <c:v>1.8403692245483398</c:v>
-                </c:pt>
-                <c:pt idx="141">
-                  <c:v>1.8370065689086914</c:v>
-                </c:pt>
-                <c:pt idx="142">
-                  <c:v>1.7377748489379883</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-19E1-48C8-A7C8-7210880D5D7F}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:smooth val="0"/>
-        <c:axId val="171710335"/>
-        <c:axId val="1522623135"/>
-      </c:lineChart>
-      <c:catAx>
-        <c:axId val="171710335"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1522623135"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="1522623135"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="171710335"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>115</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>929640</xdr:colOff>
-      <xdr:row>138</xdr:row>
-      <xdr:rowOff>118110</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7BB35564-EA77-715A-EF40-D27FFB5899CF}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -84993,6 +81882,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>